<commit_message>
Ricerca ambiziosa: filone canali; foglio «Ambizioso - cosa serve» (valori provvisori)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenari_kalab.xlsx
+++ b/scenari_kalab.xlsx
@@ -14,8 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stagionalità" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenari" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equilibrio" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Logistica" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confronto accordi" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambizioso - cosa serve" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Logistica" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confronto accordi" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,8 +25,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -99,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -131,7 +133,11 @@
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -633,6 +639,272 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Cosa succede a un ordine medio con diversi accordi (scenario medio, anno 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Accordo</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Base (lordo/netto)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Quota %</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>B2Brand per ordine (€)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Kalab margine per ordine (€)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Kalab margine % prezzo</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Commento</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>50% dell'incasso lordo (proposta di Kalab)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>lordo</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D3" s="12">
+        <f>IF(B3="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C3</f>
+        <v/>
+      </c>
+      <c r="E3" s="12">
+        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D3</f>
+        <v/>
+      </c>
+      <c r="F3" s="30">
+        <f>E3/'Conti per prodotto'!$B$10</f>
+        <v/>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Quota su merce + spedizione incassata, IVA inclusa: la lettura letterale di «50% dell'incasso».</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>50% dell'incassato netto (senza IVA, spedizione e commissioni)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>netto</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="12">
+        <f>IF(B4="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C4</f>
+        <v/>
+      </c>
+      <c r="E4" s="12">
+        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="30">
+        <f>E4/'Conti per prodotto'!$B$10</f>
+        <v/>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Stessa percentuale, base più piccola: è la prassi del settore (07 B1e).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>40% dell'incassato netto</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>netto</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D5" s="12">
+        <f>IF(B5="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C5</f>
+        <v/>
+      </c>
+      <c r="E5" s="12">
+        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="30">
+        <f>E5/'Conti per prodotto'!$B$10</f>
+        <v/>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Primo scaglione proposto: fino al rientro documentato dell'anticipo di B2Brand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>30% dell'incassato netto</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>netto</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D6" s="12">
+        <f>IF(B6="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="30">
+        <f>E6/'Conti per prodotto'!$B$10</f>
+        <v/>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Secondo scaglione, dopo il rientro. Fascia alta dell'outsourcing italiano (15-30%, 07).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>20% dell'incassato netto</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>netto</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D7" s="12">
+        <f>IF(B7="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="12">
+        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="30">
+        <f>E7/'Conti per prodotto'!$B$10</f>
+        <v/>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Terzo scaglione sopra una soglia annua. Sotto, B2Brand non copre nemmeno le ore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>10% netto sugli ordini B2B passati dal sito</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>netto</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D8" s="12">
+        <f>IF(B8="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="12">
+        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="30">
+        <f>E8/'Conti per prodotto'!$B$10</f>
+        <v/>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Per ristoranti, bar e botteghe che ordinano dal sito con listino riservato: volumi alti, margine basso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lettura: l'ordine medio è quello del foglio Conti (mix di categorie). Il margine di Kalab è dopo prodotto, imballo, spedizione vera e perdite. Per vedere l'effetto sui 36 mesi, cambiare quota e base nel foglio Ipotesi.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -9738,6 +10010,429 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Scenario ambizioso: cosa deve succedere ogni mese, a regime, per arrivarci</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Celle azzurre = valori di riferimento dai benchmark (fonte in ricerca/ambizioso/02_benchmark_e_numeri.md). Ordini e pubblicità arrivano dal foglio Scenari, colonna Ambizioso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Voce</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Anno 1</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Anno 2</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Anno 3</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tasso di conversione del sito</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C5" s="25" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D5" s="25" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tasso di conversione del sito (ordini ÷ visite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Ordini da clienti che ritornano</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C6" s="26" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>quota degli ordini fatta da clienti che hanno già comprato</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Costo di un clic a pagamento (€)</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>costo medio di un clic a pagamento (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Costo pubblicitario per un cliente nuovo (€)</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>25</v>
+      </c>
+      <c r="C8" s="27" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <v>25</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>costo pubblicitario per un cliente nuovo (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Quota degli ordini dalla newsletter</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C9" s="26" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>quota degli ordini che arriva dalla newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Ordini al mese ogni 1.000 iscritti</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ordini al mese ogni 1.000 iscritti alla newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Ordini al mese (obiettivo a regime)</t>
+        </is>
+      </c>
+      <c r="B12" s="20">
+        <f>Scenari!$D$3</f>
+        <v/>
+      </c>
+      <c r="C12" s="20">
+        <f>Scenari!$D$4</f>
+        <v/>
+      </c>
+      <c r="D12" s="20">
+        <f>Scenari!$D$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Pubblicità al mese (€)</t>
+        </is>
+      </c>
+      <c r="B13" s="20">
+        <f>Scenari!$D$7</f>
+        <v/>
+      </c>
+      <c r="C13" s="20">
+        <f>Scenari!$D$8</f>
+        <v/>
+      </c>
+      <c r="D13" s="20">
+        <f>Scenari!$D$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Visite al mese necessarie</t>
+        </is>
+      </c>
+      <c r="B14" s="20">
+        <f>ROUND(B12/B5,0)</f>
+        <v/>
+      </c>
+      <c r="C14" s="20">
+        <f>ROUND(C12/C5,0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="20">
+        <f>ROUND(D12/D5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>…di cui comprate con la pubblicità</t>
+        </is>
+      </c>
+      <c r="B15" s="20">
+        <f>ROUND(B13/B7,0)</f>
+        <v/>
+      </c>
+      <c r="C15" s="20">
+        <f>ROUND(C13/C7,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="20">
+        <f>ROUND(D13/D7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>…di cui da portare gratis (Google, social, eventi, passaparola)</t>
+        </is>
+      </c>
+      <c r="B16" s="20">
+        <f>MAX(0,B14-B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="20">
+        <f>MAX(0,C14-C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="20">
+        <f>MAX(0,D14-D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Clienti nuovi al mese</t>
+        </is>
+      </c>
+      <c r="B17" s="20">
+        <f>ROUND(B12*(1-B6),0)</f>
+        <v/>
+      </c>
+      <c r="C17" s="20">
+        <f>ROUND(C12*(1-C6),0)</f>
+        <v/>
+      </c>
+      <c r="D17" s="20">
+        <f>ROUND(D12*(1-D6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>…di cui comprati con la pubblicità</t>
+        </is>
+      </c>
+      <c r="B18" s="20">
+        <f>ROUND(B13/B8,0)</f>
+        <v/>
+      </c>
+      <c r="C18" s="20">
+        <f>ROUND(C13/C8,0)</f>
+        <v/>
+      </c>
+      <c r="D18" s="20">
+        <f>ROUND(D13/D8,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>…di cui da trovare gratis</t>
+        </is>
+      </c>
+      <c r="B19" s="20">
+        <f>MAX(0,B17-B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="20">
+        <f>MAX(0,C17-C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="20">
+        <f>MAX(0,D17-D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Ordini di clienti che ritornano</t>
+        </is>
+      </c>
+      <c r="B20" s="20">
+        <f>ROUND(B12*B6,0)</f>
+        <v/>
+      </c>
+      <c r="C20" s="20">
+        <f>ROUND(C12*C6,0)</f>
+        <v/>
+      </c>
+      <c r="D20" s="20">
+        <f>ROUND(D12*D6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Ordini dalla newsletter</t>
+        </is>
+      </c>
+      <c r="B21" s="20">
+        <f>ROUND(B12*B9,0)</f>
+        <v/>
+      </c>
+      <c r="C21" s="20">
+        <f>ROUND(C12*C9,0)</f>
+        <v/>
+      </c>
+      <c r="D21" s="20">
+        <f>ROUND(D12*D9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Iscritti alla newsletter necessari</t>
+        </is>
+      </c>
+      <c r="B22" s="20">
+        <f>ROUND(B21/B10*1000,0)</f>
+        <v/>
+      </c>
+      <c r="C22" s="20">
+        <f>ROUND(C21/C10*1000,0)</f>
+        <v/>
+      </c>
+      <c r="D22" s="20">
+        <f>ROUND(D21/D10*1000,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Ordini al giorno</t>
+        </is>
+      </c>
+      <c r="B23" s="29">
+        <f>ROUND(B12/30,1)</f>
+        <v/>
+      </c>
+      <c r="C23" s="29">
+        <f>ROUND(C12/30,1)</f>
+        <v/>
+      </c>
+      <c r="D23" s="29">
+        <f>ROUND(D12/30,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Lettura: la riga «da portare gratis» è il lavoro vero del marchio. Se è troppo alta rispetto a quello che Google, social, eventi e B2B possono dare, l'ambizioso non si raggiunge con quella pubblicità.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -10150,270 +10845,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Cosa succede a un ordine medio con diversi accordi (scenario medio, anno 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Accordo</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Base (lordo/netto)</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Quota %</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>B2Brand per ordine (€)</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Kalab margine per ordine (€)</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Kalab margine % prezzo</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Commento</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>50% dell'incasso lordo (proposta di Kalab)</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>lordo</t>
-        </is>
-      </c>
-      <c r="C3" s="25" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D3" s="12">
-        <f>IF(B3="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C3</f>
-        <v/>
-      </c>
-      <c r="E3" s="12">
-        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D3</f>
-        <v/>
-      </c>
-      <c r="F3" s="26">
-        <f>E3/'Conti per prodotto'!$B$10</f>
-        <v/>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Quota su merce + spedizione incassata, IVA inclusa: la lettura letterale di «50% dell'incasso».</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>50% dell'incassato netto (senza IVA, spedizione e commissioni)</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>netto</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D4" s="12">
-        <f>IF(B4="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C4</f>
-        <v/>
-      </c>
-      <c r="E4" s="12">
-        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D4</f>
-        <v/>
-      </c>
-      <c r="F4" s="26">
-        <f>E4/'Conti per prodotto'!$B$10</f>
-        <v/>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Stessa percentuale, base più piccola: è la prassi del settore (07 B1e).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>40% dell'incassato netto</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>netto</t>
-        </is>
-      </c>
-      <c r="C5" s="25" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D5" s="12">
-        <f>IF(B5="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C5</f>
-        <v/>
-      </c>
-      <c r="E5" s="12">
-        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D5</f>
-        <v/>
-      </c>
-      <c r="F5" s="26">
-        <f>E5/'Conti per prodotto'!$B$10</f>
-        <v/>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Primo scaglione proposto: fino al rientro documentato dell'anticipo di B2Brand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>30% dell'incassato netto</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>netto</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D6" s="12">
-        <f>IF(B6="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C6</f>
-        <v/>
-      </c>
-      <c r="E6" s="12">
-        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D6</f>
-        <v/>
-      </c>
-      <c r="F6" s="26">
-        <f>E6/'Conti per prodotto'!$B$10</f>
-        <v/>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Secondo scaglione, dopo il rientro. Fascia alta dell'outsourcing italiano (15-30%, 07).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>20% dell'incassato netto</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>netto</t>
-        </is>
-      </c>
-      <c r="C7" s="25" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D7" s="12">
-        <f>IF(B7="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="12">
-        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D7</f>
-        <v/>
-      </c>
-      <c r="F7" s="26">
-        <f>E7/'Conti per prodotto'!$B$10</f>
-        <v/>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Terzo scaglione sopra una soglia annua. Sotto, B2Brand non copre nemmeno le ore.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>10% netto sugli ordini B2B passati dal sito</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>netto</t>
-        </is>
-      </c>
-      <c r="C8" s="25" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D8" s="12">
-        <f>IF(B8="lordo",'Conti per prodotto'!$H$10,'Conti per prodotto'!$G$10)*C8</f>
-        <v/>
-      </c>
-      <c r="E8" s="12">
-        <f>'Conti per prodotto'!$O$10+'Conti per prodotto'!$I$10-D8</f>
-        <v/>
-      </c>
-      <c r="F8" s="26">
-        <f>E8/'Conti per prodotto'!$B$10</f>
-        <v/>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Per ristoranti, bar e botteghe che ordinano dal sito con listino riservato: volumi alti, margine basso.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Lettura: l'ordine medio è quello del foglio Conti (mix di categorie). Il margine di Kalab è dopo prodotto, imballo, spedizione vera e perdite. Per vedere l'effetto sui 36 mesi, cambiare quota e base nel foglio Ipotesi.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>